<commit_message>
Deploy: Update LINE groups, close welfare department, standardize duties, and generate consolidated PDFs
</commit_message>
<xml_diff>
--- a/เอกสารและรายชื่อคณะสีแสด_ปี69/แยกฝ่าย/กีฬา/รายชื่อนักกีฬาคณะสีแสด_แยกตามประเภทกีฬา_ปี69.xlsx
+++ b/เอกสารและรายชื่อคณะสีแสด_ปี69/แยกฝ่าย/กีฬา/รายชื่อนักกีฬาคณะสีแสด_แยกตามประเภทกีฬา_ปี69.xlsx
@@ -17,15 +17,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="356">
   <si>
     <t>⚽ รายชื่อนักกีฬาฝ่ายฟุตบอล — คณะสีแสด (สีบุษราคัม) ปี 2569</t>
   </si>
   <si>
-    <t>จำนวนนักกีฬาทั้งหมด 43 คน | การแข่งขันกีฬาสีภายใน ประจำปีการศึกษา 2569</t>
-  </si>
-  <si>
-    <t>▶ ทีมชาย มัธยมศึกษาตอนต้น (17 คน)</t>
+    <t>จำนวนนักกีฬาทั้งหมด 47 คน | การแข่งขันกีฬาสีภายใน ประจำปีการศึกษา 2569</t>
+  </si>
+  <si>
+    <t>▶ ทีมชาย มัธยมศึกษาตอนต้น (18 คน)</t>
   </si>
   <si>
     <t>ลำดับ</t>
@@ -187,6 +187,18 @@
     <t>เด็กชายธนวัฒน์ พรมเมือง</t>
   </si>
   <si>
+    <t>ม.3/11</t>
+  </si>
+  <si>
+    <t>34007</t>
+  </si>
+  <si>
+    <t>เด็กชายสุวิจักขณ์ กฤติโอภาสพงศ์</t>
+  </si>
+  <si>
+    <t>061-150-8435</t>
+  </si>
+  <si>
     <t>▶ ทีมชาย มัธยมศึกษาตอนปลาย (10 คน)</t>
   </si>
   <si>
@@ -280,7 +292,7 @@
     <t>นายสิปปกร ศิริวงขันธ์</t>
   </si>
   <si>
-    <t>▶ ทีมหญิง มัธยมศึกษาตอนต้น (12 คน)</t>
+    <t>▶ ทีมหญิง มัธยมศึกษาตอนต้น (14 คน)</t>
   </si>
   <si>
     <t>33725</t>
@@ -394,7 +406,25 @@
     <t>080 800 6634</t>
   </si>
   <si>
-    <t>▶ ทีมหญิง มัธยมศึกษาตอนปลาย (4 คน)</t>
+    <t>ม.2/2</t>
+  </si>
+  <si>
+    <t>34331</t>
+  </si>
+  <si>
+    <t>เด็กหญิงปณัฎฎา นาคพันธ์</t>
+  </si>
+  <si>
+    <t>34343</t>
+  </si>
+  <si>
+    <t>เด็กหญิงวัชรินทร์ ชื่นยศ</t>
+  </si>
+  <si>
+    <t>091-030-4248</t>
+  </si>
+  <si>
+    <t>▶ ทีมหญิง มัธยมศึกษาตอนปลาย (5 คน)</t>
   </si>
   <si>
     <t>ม.5/4</t>
@@ -439,10 +469,22 @@
     <t>084-989-0044</t>
   </si>
   <si>
+    <t>ม.4/7</t>
+  </si>
+  <si>
+    <t>33044</t>
+  </si>
+  <si>
+    <t>นางสาวชลธิชา พลศักดิ์</t>
+  </si>
+  <si>
+    <t>099-193-7702</t>
+  </si>
+  <si>
     <t>🏀 รายชื่อนักกีฬาฝ่ายบาสเกตบอล — คณะสีแสด (สีบุษราคัม) ปี 2569</t>
   </si>
   <si>
-    <t>จำนวนนักกีฬาทั้งหมด 15 คน | การแข่งขันกีฬาสีภายใน ประจำปีการศึกษา 2569</t>
+    <t>จำนวนนักกีฬาทั้งหมด 18 คน | การแข่งขันกีฬาสีภายใน ประจำปีการศึกษา 2569</t>
   </si>
   <si>
     <t>▶ ทีมชาย มัธยมศึกษาตอนต้น (10 คน)</t>
@@ -523,7 +565,7 @@
     <t>เด็กชายบวรรัตน์ แสนจุ้ม</t>
   </si>
   <si>
-    <t>▶ ทีมชาย มัธยมศึกษาตอนปลาย (2 คน)</t>
+    <t>▶ ทีมชาย มัธยมศึกษาตอนปลาย (3 คน)</t>
   </si>
   <si>
     <t>35512</t>
@@ -538,7 +580,19 @@
     <t>นายภูวิศ ไชยบุญเรือง</t>
   </si>
   <si>
-    <t>▶ ทีมหญิง (ม.ต้น) (3 คน)</t>
+    <t>ม.6/3</t>
+  </si>
+  <si>
+    <t>31816</t>
+  </si>
+  <si>
+    <t>นายธนกฤต อรุณเกล้า</t>
+  </si>
+  <si>
+    <t>082-590-6971</t>
+  </si>
+  <si>
+    <t>▶ ทีมหญิง (ม.ต้น) (5 คน)</t>
   </si>
   <si>
     <t>ม.2/5</t>
@@ -565,6 +619,12 @@
     <t>เด็กหญิงณัฐธิดา วรรณิน</t>
   </si>
   <si>
+    <t>061-983-7797</t>
+  </si>
+  <si>
+    <t>093-131-8108</t>
+  </si>
+  <si>
     <t>🏐 รายชื่อนักกีฬาฝ่ายวอลเลย์บอล — คณะสีแสด (สีบุษราคัม) ปี 2569</t>
   </si>
   <si>
@@ -589,9 +649,6 @@
     <t>เด็กชายอติเทพ สิงห์คา</t>
   </si>
   <si>
-    <t>ม.2/2</t>
-  </si>
-  <si>
     <t>34307</t>
   </si>
   <si>
@@ -634,24 +691,12 @@
     <t>เด็กหญิงเพชรลดา คำลือเมือง</t>
   </si>
   <si>
-    <t>34331</t>
-  </si>
-  <si>
-    <t>เด็กหญิงปณัฎฎา นาคพันธ์</t>
-  </si>
-  <si>
     <t>34337</t>
   </si>
   <si>
     <t>เด็กหญิงภัทรสุดา สุนทรปาน</t>
   </si>
   <si>
-    <t>34343</t>
-  </si>
-  <si>
-    <t>เด็กหญิงวัชรินทร์ ชื่นยศ</t>
-  </si>
-  <si>
     <t>33773</t>
   </si>
   <si>
@@ -697,9 +742,6 @@
     <t>▶ ทีมหญิง มัธยมศึกษาตอนปลาย (2 คน)</t>
   </si>
   <si>
-    <t>ม.4/7</t>
-  </si>
-  <si>
     <t>35490</t>
   </si>
   <si>
@@ -772,10 +814,10 @@
     <t>⚪ รายชื่อนักกีฬาฝ่ายเปตอง — คณะสีแสด (สีบุษราคัม) ปี 2569</t>
   </si>
   <si>
-    <t>จำนวนนักกีฬาทั้งหมด 11 คน | การแข่งขันกีฬาสีภายใน ประจำปีการศึกษา 2569</t>
-  </si>
-  <si>
-    <t>▶ ทีม มัธยมศึกษาตอนต้น (ชาย/หญิง) (10 คน)</t>
+    <t>จำนวนนักกีฬาทั้งหมด 12 คน | การแข่งขันกีฬาสีภายใน ประจำปีการศึกษา 2569</t>
+  </si>
+  <si>
+    <t>▶ ทีม มัธยมศึกษาตอนต้น (ชาย/หญิง) (11 คน)</t>
   </si>
   <si>
     <t>34349</t>
@@ -832,6 +874,15 @@
     <t>เด็กหญิงนฐมนพรรณ เขื่อนวิชัย</t>
   </si>
   <si>
+    <t>34301</t>
+  </si>
+  <si>
+    <t>เด็กหญิงมัณฑิตา เนตรแก้ว</t>
+  </si>
+  <si>
+    <t>098-567-1827</t>
+  </si>
+  <si>
     <t>33160</t>
   </si>
   <si>
@@ -844,10 +895,7 @@
     <t>🏃 รายชื่อนักกีฬาฝ่ายกรีฑา — คณะสีแสด (สีบุษราคัม) ปี 2569</t>
   </si>
   <si>
-    <t>จำนวนนักกีฬาทั้งหมด 10 คน | การแข่งขันกีฬาสีภายใน ประจำปีการศึกษา 2569</t>
-  </si>
-  <si>
-    <t>▶ ทีม มัธยมศึกษาตอนต้น (ชาย/หญิง) (8 คน)</t>
+    <t>จำนวนนักกีฬาทั้งหมด 14 คน | การแข่งขันกีฬาสีภายใน ประจำปีการศึกษา 2569</t>
   </si>
   <si>
     <t>34271</t>
@@ -904,7 +952,16 @@
     <t>082 307 8878</t>
   </si>
   <si>
-    <t>▶ ทีม มัธยมศึกษาตอนปลาย (ชาย/หญิง) (2 คน)</t>
+    <t>33827</t>
+  </si>
+  <si>
+    <t>นายวีรศักดิ์ วงศ์หิรัญวเรศ</t>
+  </si>
+  <si>
+    <t>061-439-7907</t>
+  </si>
+  <si>
+    <t>▶ ทีม มัธยมศึกษาตอนปลาย (ชาย/หญิง) (3 คน)</t>
   </si>
   <si>
     <t>ม.4/14</t>
@@ -919,10 +976,19 @@
     <t>099 462 8457</t>
   </si>
   <si>
+    <t>32394</t>
+  </si>
+  <si>
+    <t>นายกษิดิศ ปันทิ</t>
+  </si>
+  <si>
     <t>🏃‍♂️🏃‍♀️ รายชื่อนักกีฬาฝ่ายวิ่ง 16 ขา — คณะสีแสด (สีบุษราคัม) ปี 2569</t>
   </si>
   <si>
-    <t>▶ ทีมชาย มัธยมศึกษาตอนปลาย (4 คน)</t>
+    <t>จำนวนนักกีฬาทั้งหมด 13 คน | การแข่งขันกีฬาสีภายใน ประจำปีการศึกษา 2569</t>
+  </si>
+  <si>
+    <t>▶ ทีมชาย มัธยมศึกษาตอนปลาย (6 คน)</t>
   </si>
   <si>
     <t>35461</t>
@@ -962,6 +1028,24 @@
   </si>
   <si>
     <t>093-329-6478</t>
+  </si>
+  <si>
+    <t>35455</t>
+  </si>
+  <si>
+    <t>นายนรภัทร ขัตติยะวงษ์</t>
+  </si>
+  <si>
+    <t>099-435-6995</t>
+  </si>
+  <si>
+    <t>35500</t>
+  </si>
+  <si>
+    <t>นายธัญสิทธิ์ กิจสุวรรณ</t>
+  </si>
+  <si>
+    <t>083-214-0843</t>
   </si>
   <si>
     <t>▶ ทีมหญิง มัธยมศึกษาตอนปลาย (7 คน)</t>
@@ -1485,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1945,703 +2029,795 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+    <row r="23" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="7">
+        <v>18</v>
+      </c>
+      <c r="B23" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
+      <c r="C23" s="7">
+        <v>12</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="25" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+    </row>
+    <row r="26" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B26" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C26" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D26" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E26" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F26" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G26" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="5">
+    <row r="27" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
         <v>1</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C26" s="5">
-        <v>13</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="7">
+      <c r="B27" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="5">
+        <v>13</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="7">
         <v>2</v>
       </c>
-      <c r="B27" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="C27" s="7">
+      <c r="B28" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" s="7">
         <v>5</v>
       </c>
-      <c r="D27" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="5">
+      <c r="D28" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
         <v>3</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="5">
+      <c r="B29" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" s="5">
         <v>3</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="7">
+      <c r="D29" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="7">
         <v>4</v>
       </c>
-      <c r="B29" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="C29" s="7">
-        <v>13</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="5">
+      <c r="B30" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30" s="7">
+        <v>13</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
         <v>5</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C30" s="5">
+      <c r="B31" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C31" s="5">
         <v>11</v>
       </c>
-      <c r="D30" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="7">
+      <c r="D31" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="7">
         <v>6</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="C31" s="7">
+      <c r="B32" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C32" s="7">
         <v>7</v>
       </c>
-      <c r="D31" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="5">
+      <c r="D32" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
         <v>7</v>
       </c>
-      <c r="B32" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C32" s="5">
+      <c r="B33" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" s="5">
         <v>12</v>
       </c>
-      <c r="D32" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="7">
+      <c r="D33" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="7">
         <v>8</v>
       </c>
-      <c r="B33" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C33" s="7">
+      <c r="B34" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" s="7">
         <v>12</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D34" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="5">
+        <v>9</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C35" s="5">
+        <v>7</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="7">
+        <v>10</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E33" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="G33" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="5">
+      <c r="C36" s="7">
+        <v>17</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+    </row>
+    <row r="39" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G39" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C34" s="5">
+    </row>
+    <row r="40" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="5">
+        <v>1</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C40" s="5">
+        <v>33</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="7">
+        <v>2</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C41" s="7">
+        <v>21</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="5">
+        <v>3</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C42" s="5">
+        <v>26</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="7">
+        <v>4</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C43" s="7">
+        <v>22</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="5">
+        <v>5</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="5">
+        <v>40</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="7">
+        <v>6</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="7">
+        <v>22</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="G45" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="5">
         <v>7</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="7">
+      <c r="B46" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C46" s="5">
+        <v>21</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="7">
+        <v>8</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C47" s="7">
+        <v>27</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="5">
+        <v>9</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C48" s="5">
+        <v>40</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="7">
         <v>10</v>
       </c>
-      <c r="B35" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C35" s="7">
+      <c r="B49" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C49" s="7">
+        <v>24</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G49" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="5">
+        <v>11</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C50" s="5">
+        <v>30</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="7">
+        <v>12</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C51" s="7">
+        <v>25</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="5">
+        <v>13</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C52" s="5">
+        <v>37</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="F52" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="7">
+        <v>14</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C53" s="7">
+        <v>21</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+    </row>
+    <row r="56" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="5">
+        <v>1</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C57" s="5">
+        <v>30</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="7">
+        <v>2</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C58" s="7">
+        <v>23</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="G58" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="5">
+        <v>3</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C59" s="5">
         <v>17</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-    </row>
-    <row r="38" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B38" s="4" t="s">
+      <c r="D59" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="G59" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="7">
         <v>4</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="B60" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C60" s="7">
+        <v>36</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="F60" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="G60" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="5">
         <v>5</v>
       </c>
-      <c r="D38" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="39" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="5">
-        <v>1</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C39" s="5">
-        <v>33</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="7">
-        <v>2</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C40" s="7">
-        <v>21</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="G40" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="41" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="5">
-        <v>3</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C41" s="5">
-        <v>26</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="G41" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="7">
-        <v>4</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C42" s="7">
-        <v>22</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="G42" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="43" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="5">
-        <v>5</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C43" s="5">
-        <v>40</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="7">
-        <v>6</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" s="7">
-        <v>22</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="E44" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="G44" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="5">
-        <v>7</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C45" s="5">
-        <v>21</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="G45" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="7">
-        <v>8</v>
-      </c>
-      <c r="B46" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C46" s="7">
-        <v>27</v>
-      </c>
-      <c r="D46" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F46" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="G46" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="47" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="5">
-        <v>9</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="C47" s="5">
-        <v>40</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="48" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="7">
-        <v>10</v>
-      </c>
-      <c r="B48" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="C48" s="7">
-        <v>24</v>
-      </c>
-      <c r="D48" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="E48" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="F48" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="G48" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="5">
-        <v>11</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="C49" s="5">
-        <v>30</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="G49" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="7">
-        <v>12</v>
-      </c>
-      <c r="B50" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C50" s="7">
-        <v>21</v>
-      </c>
-      <c r="D50" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E50" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G50" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="52" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="3"/>
-    </row>
-    <row r="53" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F53" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="G53" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="54" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="5">
-        <v>1</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C54" s="5">
-        <v>30</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="F54" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="G54" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="55" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="7">
-        <v>2</v>
-      </c>
-      <c r="B55" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="C55" s="7">
-        <v>23</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="E55" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="F55" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="G55" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="56" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="5">
-        <v>3</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="C56" s="5">
+      <c r="B61" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C61" s="5">
         <v>17</v>
       </c>
-      <c r="D56" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="F56" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="G56" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="57" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="7">
-        <v>4</v>
-      </c>
-      <c r="B57" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="C57" s="7">
-        <v>36</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="E57" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="F57" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="G57" s="7" t="s">
+      <c r="D61" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="F61" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="G61" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -2650,9 +2826,9 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A37:G37"/>
-    <mergeCell ref="A52:G52"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A55:G55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2661,7 +2837,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2675,7 +2851,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2686,7 +2862,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2698,7 +2874,7 @@
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -2741,10 +2917,10 @@
         <v>10</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>13</v>
@@ -2764,10 +2940,10 @@
         <v>17</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>13</v>
@@ -2781,16 +2957,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="C8" s="5">
         <v>7</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>13</v>
@@ -2810,10 +2986,10 @@
         <v>26</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>13</v>
@@ -2827,16 +3003,16 @@
         <v>5</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="C10" s="5">
         <v>2</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>13</v>
@@ -2850,19 +3026,19 @@
         <v>6</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="C11" s="7">
         <v>6</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>14</v>
@@ -2873,16 +3049,16 @@
         <v>7</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C12" s="5">
         <v>4</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>13</v>
@@ -2896,16 +3072,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="C13" s="7">
         <v>6</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>13</v>
@@ -2919,16 +3095,16 @@
         <v>9</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C14" s="5">
         <v>10</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>13</v>
@@ -2948,10 +3124,10 @@
         <v>10</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>13</v>
@@ -2962,7 +3138,7 @@
     </row>
     <row r="17" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -2999,16 +3175,16 @@
         <v>1</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C19" s="5">
         <v>9</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>13</v>
@@ -3022,16 +3198,16 @@
         <v>2</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C20" s="7">
         <v>1</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>13</v>
@@ -3040,106 +3216,175 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
+    <row r="21" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
+        <v>3</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="C21" s="5">
+        <v>5</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="23" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+    </row>
+    <row r="24" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B24" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C24" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E24" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F24" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G24" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="5">
+    <row r="25" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
         <v>1</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="C24" s="5">
+      <c r="B25" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="C25" s="5">
         <v>22</v>
       </c>
-      <c r="D24" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="7">
+      <c r="D25" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="7">
         <v>2</v>
       </c>
-      <c r="B25" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="C25" s="7">
+      <c r="B26" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="C26" s="7">
         <v>27</v>
       </c>
-      <c r="D25" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="5">
+      <c r="D26" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
         <v>3</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="C26" s="5">
+      <c r="B27" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="C27" s="5">
         <v>24</v>
       </c>
-      <c r="D26" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="5" t="s">
+      <c r="D27" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="7">
+        <v>4</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="7">
+        <v>33</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>5</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C29" s="5">
+        <v>24</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="G29" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -3149,7 +3394,7 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -3172,7 +3417,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>202</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3183,7 +3428,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3195,7 +3440,7 @@
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -3232,16 +3477,16 @@
         <v>1</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="C6" s="5">
         <v>5</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>13</v>
@@ -3255,16 +3500,16 @@
         <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="C7" s="7">
         <v>11</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>189</v>
+        <v>209</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>13</v>
@@ -3278,16 +3523,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>190</v>
+        <v>129</v>
       </c>
       <c r="C8" s="5">
         <v>1</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>13</v>
@@ -3301,16 +3546,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>190</v>
+        <v>129</v>
       </c>
       <c r="C9" s="7">
         <v>13</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>13</v>
@@ -3330,10 +3575,10 @@
         <v>15</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>196</v>
+        <v>215</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>13</v>
@@ -3347,19 +3592,19 @@
         <v>6</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="C11" s="7">
         <v>7</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>14</v>
@@ -3367,7 +3612,7 @@
     </row>
     <row r="13" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -3404,16 +3649,16 @@
         <v>1</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
       <c r="C15" s="5">
         <v>40</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>13</v>
@@ -3427,16 +3672,16 @@
         <v>2</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>190</v>
+        <v>129</v>
       </c>
       <c r="C16" s="7">
         <v>25</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>205</v>
+        <v>130</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>206</v>
+        <v>131</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>13</v>
@@ -3450,16 +3695,16 @@
         <v>3</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>190</v>
+        <v>129</v>
       </c>
       <c r="C17" s="5">
         <v>31</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>207</v>
+        <v>224</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>13</v>
@@ -3473,16 +3718,16 @@
         <v>4</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>190</v>
+        <v>129</v>
       </c>
       <c r="C18" s="7">
         <v>37</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>209</v>
+        <v>132</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>210</v>
+        <v>133</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>13</v>
@@ -3502,10 +3747,10 @@
         <v>40</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>13</v>
@@ -3525,10 +3770,10 @@
         <v>22</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>13</v>
@@ -3548,10 +3793,10 @@
         <v>21</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>13</v>
@@ -3565,16 +3810,16 @@
         <v>8</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="C22" s="7">
         <v>40</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>13</v>
@@ -3585,7 +3830,7 @@
     </row>
     <row r="24" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -3622,16 +3867,16 @@
         <v>1</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C26" s="5">
         <v>7</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>215</v>
+        <v>230</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>13</v>
@@ -3645,16 +3890,16 @@
         <v>2</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C27" s="7">
         <v>25</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>13</v>
@@ -3668,16 +3913,16 @@
         <v>3</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C28" s="5">
         <v>9</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="F28" s="5" t="s">
         <v>13</v>
@@ -3691,19 +3936,19 @@
         <v>4</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C29" s="7">
         <v>17</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="G29" s="7" t="s">
         <v>14</v>
@@ -3714,19 +3959,19 @@
         <v>5</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
       <c r="C30" s="5">
         <v>7</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>14</v>
@@ -3734,7 +3979,7 @@
     </row>
     <row r="32" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -3771,16 +4016,16 @@
         <v>1</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>226</v>
+        <v>150</v>
       </c>
       <c r="C34" s="5">
         <v>35</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>13</v>
@@ -3794,19 +4039,19 @@
         <v>2</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C35" s="7">
         <v>37</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
       <c r="G35" s="7" t="s">
         <v>14</v>
@@ -3842,7 +4087,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3853,7 +4098,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3865,7 +4110,7 @@
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -3914,7 +4159,7 @@
         <v>51</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>14</v>
@@ -3937,7 +4182,7 @@
         <v>49</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>14</v>
@@ -3945,7 +4190,7 @@
     </row>
     <row r="9" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -3982,19 +4227,19 @@
         <v>1</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C11" s="5">
         <v>25</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>14</v>
@@ -4005,19 +4250,19 @@
         <v>2</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="C12" s="7">
         <v>8</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>14</v>
@@ -4028,16 +4273,16 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="C13" s="5">
         <v>4</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>13</v>
@@ -4051,19 +4296,19 @@
         <v>4</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="C14" s="7">
         <v>21</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>245</v>
+        <v>259</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>246</v>
+        <v>260</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>247</v>
+        <v>261</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>14</v>
@@ -4074,19 +4319,19 @@
         <v>5</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="C15" s="5">
         <v>10</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>249</v>
+        <v>263</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>14</v>
@@ -4106,7 +4351,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -4120,7 +4365,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4131,7 +4376,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>251</v>
+        <v>265</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4143,7 +4388,7 @@
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -4186,10 +4431,10 @@
         <v>3</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>13</v>
@@ -4209,10 +4454,10 @@
         <v>27</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>255</v>
+        <v>269</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>13</v>
@@ -4232,10 +4477,10 @@
         <v>7</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>257</v>
+        <v>271</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>13</v>
@@ -4255,10 +4500,10 @@
         <v>37</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>13</v>
@@ -4272,16 +4517,16 @@
         <v>5</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C10" s="5">
         <v>6</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>13</v>
@@ -4295,16 +4540,16 @@
         <v>6</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="C11" s="7">
         <v>21</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>13</v>
@@ -4318,16 +4563,16 @@
         <v>7</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="C12" s="5">
         <v>12</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>13</v>
@@ -4341,16 +4586,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="C13" s="7">
         <v>24</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>268</v>
+        <v>282</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>13</v>
@@ -4370,10 +4615,10 @@
         <v>17</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>269</v>
+        <v>283</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>270</v>
+        <v>284</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>13</v>
@@ -4387,78 +4632,101 @@
         <v>10</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="C15" s="7">
+        <v>36</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="5">
+        <v>11</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="5">
         <v>7</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
+      <c r="D16" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="18" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+    </row>
+    <row r="19" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F19" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G19" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="5">
+    <row r="20" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="5">
         <v>1</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C19" s="5">
+      <c r="B20" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="5">
         <v>7</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="5" t="s">
+      <c r="D20" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -4467,7 +4735,7 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4476,7 +4744,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -4490,7 +4758,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>274</v>
+        <v>291</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4501,7 +4769,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>275</v>
+        <v>292</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4513,7 +4781,7 @@
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -4556,13 +4824,13 @@
         <v>5</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>277</v>
+        <v>293</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>278</v>
+        <v>294</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>14</v>
@@ -4579,13 +4847,13 @@
         <v>9</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>280</v>
+        <v>296</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>281</v>
+        <v>297</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>282</v>
+        <v>298</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>14</v>
@@ -4596,19 +4864,19 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="C8" s="5">
         <v>11</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>189</v>
+        <v>209</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>283</v>
+        <v>299</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>14</v>
@@ -4625,13 +4893,13 @@
         <v>27</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>284</v>
+        <v>300</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>14</v>
@@ -4642,19 +4910,19 @@
         <v>5</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="C10" s="5">
         <v>7</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>14</v>
@@ -4665,19 +4933,19 @@
         <v>6</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="C11" s="7">
         <v>33</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>286</v>
+        <v>302</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>287</v>
+        <v>303</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>14</v>
@@ -4688,19 +4956,19 @@
         <v>7</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>288</v>
+        <v>304</v>
       </c>
       <c r="C12" s="5">
         <v>28</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>289</v>
+        <v>305</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>290</v>
+        <v>306</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>291</v>
+        <v>307</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>14</v>
@@ -4711,101 +4979,193 @@
         <v>8</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>288</v>
+        <v>304</v>
       </c>
       <c r="C13" s="7">
         <v>39</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>292</v>
+        <v>308</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>293</v>
+        <v>309</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>294</v>
+        <v>310</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-    </row>
-    <row r="16" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+    <row r="14" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>9</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="5">
+        <v>33</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="7">
+        <v>10</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C15" s="7">
+        <v>12</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="5">
+        <v>11</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C16" s="5">
+        <v>24</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+    </row>
+    <row r="19" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F19" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G19" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="5">
+    <row r="20" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="5">
         <v>1</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="5">
+      <c r="B20" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="5">
         <v>37</v>
       </c>
-      <c r="D17" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="7">
+      <c r="D20" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="7">
         <v>2</v>
       </c>
-      <c r="B18" s="7" t="s">
-        <v>296</v>
-      </c>
-      <c r="C18" s="7">
+      <c r="B21" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="C21" s="7">
         <v>11</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>297</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>298</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>299</v>
-      </c>
-      <c r="G18" s="7" t="s">
+      <c r="D21" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="5">
+        <v>3</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C22" s="5">
+        <v>2</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -4814,7 +5174,7 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A18:G18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4823,7 +5183,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -4837,7 +5197,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>300</v>
+        <v>321</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4848,7 +5208,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>251</v>
+        <v>322</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4860,7 +5220,7 @@
     <row r="3" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>301</v>
+        <v>323</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -4897,19 +5257,19 @@
         <v>1</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C6" s="5">
         <v>37</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>302</v>
+        <v>324</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>303</v>
+        <v>325</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>304</v>
+        <v>326</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>14</v>
@@ -4920,19 +5280,19 @@
         <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>305</v>
+        <v>327</v>
       </c>
       <c r="C7" s="7">
         <v>5</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>306</v>
+        <v>328</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>307</v>
+        <v>329</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>14</v>
@@ -4943,19 +5303,19 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>305</v>
+        <v>327</v>
       </c>
       <c r="C8" s="5">
         <v>17</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>310</v>
+        <v>332</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>311</v>
+        <v>333</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>14</v>
@@ -4966,122 +5326,122 @@
         <v>4</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="C9" s="7">
         <v>5</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>312</v>
+        <v>334</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>313</v>
+        <v>335</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>314</v>
+        <v>336</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-    </row>
-    <row r="12" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="10" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
+        <v>5</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="5">
+        <v>13</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="7">
+        <v>6</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="7">
+        <v>19</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>341</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+    </row>
+    <row r="14" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B14" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G14" s="4" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="5">
-        <v>1</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" s="5">
-        <v>30</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>316</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>317</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="7">
-        <v>2</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="C14" s="7">
-        <v>23</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>319</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>320</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>321</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C15" s="5">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>229</v>
+        <v>344</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>230</v>
+        <v>345</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>231</v>
+        <v>346</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>14</v>
@@ -5089,22 +5449,22 @@
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>296</v>
+        <v>150</v>
       </c>
       <c r="C16" s="7">
         <v>23</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>322</v>
+        <v>347</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>323</v>
+        <v>348</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>324</v>
+        <v>349</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>14</v>
@@ -5112,22 +5472,22 @@
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C17" s="5">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>325</v>
+        <v>243</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>326</v>
+        <v>244</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>327</v>
+        <v>245</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>14</v>
@@ -5135,22 +5495,22 @@
     </row>
     <row r="18" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>72</v>
+        <v>315</v>
       </c>
       <c r="C18" s="7">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>302</v>
+        <v>350</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>303</v>
+        <v>351</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>304</v>
+        <v>352</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>14</v>
@@ -5158,24 +5518,70 @@
     </row>
     <row r="19" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
+        <v>5</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="5">
+        <v>25</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="7">
+        <v>6</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="7">
+        <v>37</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
         <v>7</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="C19" s="5">
+      <c r="B21" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C21" s="5">
         <v>35</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="G19" s="5" t="s">
+      <c r="D21" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="G21" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -5184,7 +5590,7 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A13:G13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>